<commit_message>
-Fix checker for empty values
</commit_message>
<xml_diff>
--- a/Process/Sharedpointrequest/Request/Processing.xlsx
+++ b/Process/Sharedpointrequest/Request/Processing.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\RPA Folders\Migration\Fusion_TAXLineUpdate\content\Process\Sharedpointrequest\Request\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C017E14-91D0-45BB-9124-F136EBEFBE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D33AAC7C-7584-4BEE-9F8E-1C243B2127D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7309F474-19F9-4D39-92D5-F7CF120C5A36}"/>
+    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{7309F474-19F9-4D39-92D5-F7CF120C5A36}"/>
   </bookViews>
   <sheets>
     <sheet name="Processing" sheetId="1" r:id="rId1"/>
@@ -80,13 +80,13 @@
     <t>Normal</t>
   </si>
   <si>
-    <t>LN</t>
+    <t>ELS</t>
   </si>
   <si>
     <t>Fusion_TaxLineUpdate</t>
   </si>
   <si>
-    <t>Transfer tax to address line level</t>
+    <t>Add Tax Registration Numbers</t>
   </si>
   <si>
     <t>Not Started</t>
@@ -95,7 +95,7 @@
     <t>Chua, Charles Bryan (REPH-CON)</t>
   </si>
   <si>
-    <t>ExcelTemplate_TaxUpdate_FR_0820.xlsx</t>
+    <t>ExcelTemplate_TaxUpdate_FR_1022.xlsx</t>
   </si>
   <si>
     <t>Item</t>
@@ -1120,7 +1120,7 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="7">
-        <v>8052</v>
+        <v>11167</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>13</v>
@@ -1138,7 +1138,7 @@
         <v>17</v>
       </c>
       <c r="G2" s="9">
-        <v>46254.835416666669</v>
+        <v>46317.915972222225</v>
       </c>
       <c r="H2" s="8" t="s">
         <v>18</v>
@@ -1154,11 +1154,11 @@
       </c>
       <c r="L2" s="1" t="str">
         <f>IF(A2="","",_xlfn.CONCAT("https://reedelsevier.sharepoint.com/sites/OG-P2PHdesk/Lists/RequestList/Attachments/",A2,"/",I2,"?web=1"))</f>
-        <v>https://reedelsevier.sharepoint.com/sites/OG-P2PHdesk/Lists/RequestList/Attachments/8052/ExcelTemplate_TaxUpdate_FR_0820.xlsx?web=1</v>
+        <v>https://reedelsevier.sharepoint.com/sites/OG-P2PHdesk/Lists/RequestList/Attachments/11167/ExcelTemplate_TaxUpdate_FR_1022.xlsx?web=1</v>
       </c>
       <c r="M2" s="1" t="str">
         <f>IF(A2="","",_xlfn.CONCAT("https://reedelsevier.sharepoint.com/sites/OG-P2PHdesk/Lists/RequestList/DispForm.aspx?ID=",A2))</f>
-        <v>https://reedelsevier.sharepoint.com/sites/OG-P2PHdesk/Lists/RequestList/DispForm.aspx?ID=8052</v>
+        <v>https://reedelsevier.sharepoint.com/sites/OG-P2PHdesk/Lists/RequestList/DispForm.aspx?ID=11167</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>